<commit_message>
Add enum and bitfield parser
</commit_message>
<xml_diff>
--- a/Dataframe.xlsx
+++ b/Dataframe.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Revision" sheetId="4" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>Path</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -65,6 +65,82 @@
   </si>
   <si>
     <t>Blob</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Name</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Text</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Value</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Item</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ENABLED</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DISABLED</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ENABLE_STATUS</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>VALID_STATUS</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Disabled</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Enabled</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>INVALID</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>VALID</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Invalid</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Valid</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CONNECTION_STATUS</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DISCONNECTED</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AUTHENTICATING</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AUTHENTICATION_FAILED</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CONNECTED</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -489,11 +565,124 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="29.77734375" customWidth="1"/>
+    <col min="2" max="2" width="13.44140625" customWidth="1"/>
+    <col min="3" max="3" width="29.109375" customWidth="1"/>
+    <col min="4" max="4" width="38.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B7">
+        <v>0</v>
+      </c>
+      <c r="C7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B10">
+        <v>0</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B11">
+        <v>1</v>
+      </c>
+      <c r="C11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B12">
+        <v>2</v>
+      </c>
+      <c r="C12" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>29</v>
+      </c>
+    </row>
+  </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Update and test array path expand.
</commit_message>
<xml_diff>
--- a/Dataframe.xlsx
+++ b/Dataframe.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="41">
   <si>
     <t>Path</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -141,6 +141,47 @@
   </si>
   <si>
     <t>CONNECTED</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>/Device/Engine[10]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>The engine power</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Power</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>UINT16</t>
+  </si>
+  <si>
+    <t>COMMON</t>
+  </si>
+  <si>
+    <t>MEASUREMENT</t>
+  </si>
+  <si>
+    <t>Temperature</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>/Device/Engine[10]/ControlBoard</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Voltage</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>The engine control board voltage</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>The engine control board temperature</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -495,13 +536,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="8.6640625" style="3"/>
-    <col min="3" max="3" width="16.109375" style="3" customWidth="1"/>
-    <col min="4" max="5" width="8.6640625" style="3"/>
-    <col min="6" max="6" width="9.21875" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.88671875" style="3" customWidth="1"/>
+    <col min="2" max="2" width="14.77734375" style="3" customWidth="1"/>
+    <col min="3" max="3" width="36.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.6640625" style="3"/>
+    <col min="5" max="5" width="13.6640625" style="3" customWidth="1"/>
+    <col min="6" max="6" width="11" style="3" bestFit="1" customWidth="1"/>
     <col min="7" max="9" width="8.6640625" style="3"/>
     <col min="10" max="10" width="8.6640625" style="3" customWidth="1"/>
     <col min="11" max="11" width="20.6640625" style="3" customWidth="1"/>
@@ -540,6 +583,75 @@
       </c>
       <c r="K1" s="2" t="s">
         <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E2" s="3">
+        <v>1</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E3" s="3">
+        <v>1</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E4" s="3">
+        <v>1</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Finish the row expand and path joining feature.
</commit_message>
<xml_diff>
--- a/Dataframe.xlsx
+++ b/Dataframe.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Revision" sheetId="4" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="49">
   <si>
     <t>Path</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -144,18 +144,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>/Device/Engine[10]</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>The engine power</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Power</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>UINT16</t>
   </si>
   <si>
@@ -165,24 +153,65 @@
     <t>MEASUREMENT</t>
   </si>
   <si>
-    <t>Temperature</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>/Device/Engine[10]/ControlBoard</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Voltage</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>The engine control board voltage</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>The engine control board temperature</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+    <t>/Device/SubDevice[10]/Measurement</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>/Device/SubDevice[10]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ENUM</t>
+  </si>
+  <si>
+    <t>STATUS</t>
+  </si>
+  <si>
+    <t>The sub deivce power</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Current</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>The voltage of sub device</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>The current of sub device</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>/Device/SubDevice[10]/Measurement</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>/Device/SubDevice[10]/Modules[6]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PresentStatus</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PresentStatus</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>/Device/SubDevice[10]/Modules[6]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RunningStatus</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BITFIELD</t>
   </si>
 </sst>
 </file>
@@ -526,7 +555,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -536,21 +565,21 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K4"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:K8"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="33.88671875" style="3" customWidth="1"/>
-    <col min="2" max="2" width="14.77734375" style="3" customWidth="1"/>
-    <col min="3" max="3" width="36.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.9140625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="14.75" style="3" customWidth="1"/>
+    <col min="3" max="3" width="36.58203125" style="3" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8.6640625" style="3"/>
-    <col min="5" max="5" width="13.6640625" style="3" customWidth="1"/>
-    <col min="6" max="6" width="11" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.58203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.6640625" style="3" bestFit="1" customWidth="1"/>
     <col min="7" max="9" width="8.6640625" style="3"/>
     <col min="10" max="10" width="8.6640625" style="3" customWidth="1"/>
-    <col min="11" max="11" width="20.6640625" style="3" customWidth="1"/>
+    <col min="11" max="11" width="14.08203125" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -585,73 +614,153 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="E2" s="3">
+        <v>1</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E3" s="3">
+        <v>1</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="K3" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="3" t="s">
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E4" s="3">
+        <v>1</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="K4" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E5" s="3">
+        <v>1</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E6" s="3">
+        <v>1</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="E2" s="3">
-        <v>1</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="K2" s="3" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="C3" s="3" t="s">
+      <c r="D7" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E7" s="3">
+        <v>1</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="K7" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E3" s="3">
-        <v>1</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E4" s="3">
-        <v>1</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="K4" s="3" t="s">
-        <v>35</v>
+      <c r="D8" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E8" s="3">
+        <v>1</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -678,15 +787,15 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D13"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="29.77734375" customWidth="1"/>
-    <col min="2" max="2" width="13.44140625" customWidth="1"/>
-    <col min="3" max="3" width="29.109375" customWidth="1"/>
-    <col min="4" max="4" width="38.44140625" customWidth="1"/>
+    <col min="1" max="1" width="29.75" customWidth="1"/>
+    <col min="2" max="2" width="13.4140625" customWidth="1"/>
+    <col min="3" max="3" width="29.08203125" customWidth="1"/>
+    <col min="4" max="4" width="38.4140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>11</v>
       </c>
@@ -700,12 +809,12 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B3">
         <v>0</v>
       </c>
@@ -716,7 +825,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B4">
         <v>1</v>
       </c>
@@ -727,12 +836,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B7">
         <v>0</v>
       </c>
@@ -743,7 +852,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B8">
         <v>1</v>
       </c>
@@ -754,12 +863,12 @@
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B10">
         <v>0</v>
       </c>
@@ -767,7 +876,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B11">
         <v>1</v>
       </c>
@@ -775,7 +884,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B12">
         <v>2</v>
       </c>
@@ -783,7 +892,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B13">
         <v>3</v>
       </c>
@@ -801,7 +910,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Draftly add enum generation.
</commit_message>
<xml_diff>
--- a/Dataframe.xlsx
+++ b/Dataframe.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Revision" sheetId="4" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="58">
   <si>
     <t>Path</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -84,134 +84,170 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>ENABLED</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>DISABLED</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+    <t>VALID_STATUS</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Disabled</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Enabled</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Invalid</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Valid</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CONNECTION_STATUS</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>UINT16</t>
+  </si>
+  <si>
+    <t>COMMON</t>
+  </si>
+  <si>
+    <t>MEASUREMENT</t>
+  </si>
+  <si>
+    <t>Voltage</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>/Device/SubDevice[10]/Measurement</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>/Device/SubDevice[10]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ENUM</t>
+  </si>
+  <si>
+    <t>STATUS</t>
+  </si>
+  <si>
+    <t>The sub deivce power</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Current</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>The voltage of sub device</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>The current of sub device</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>/Device/SubDevice[10]/Measurement</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>/Device/SubDevice[10]/Modules[6]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PresentStatus</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PresentStatus</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>/Device/SubDevice[10]/Modules[6]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RunningStatus</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BITFIELD</t>
   </si>
   <si>
     <t>ENABLE_STATUS</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>VALID_STATUS</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Disabled</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Enabled</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>INVALID</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>VALID</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Invalid</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Valid</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>CONNECTION_STATUS</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>DISCONNECTED</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>AUTHENTICATING</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>AUTHENTICATION_FAILED</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>CONNECTED</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>UINT16</t>
-  </si>
-  <si>
-    <t>COMMON</t>
-  </si>
-  <si>
-    <t>MEASUREMENT</t>
-  </si>
-  <si>
-    <t>Voltage</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>/Device/SubDevice[10]/Measurement</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>/Device/SubDevice[10]</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>ENUM</t>
-  </si>
-  <si>
-    <t>STATUS</t>
-  </si>
-  <si>
-    <t>The sub deivce power</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Current</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>The voltage of sub device</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>The current of sub device</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>/Device/SubDevice[10]/Measurement</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>/Device/SubDevice[10]/Modules[6]</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>PresentStatus</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>PresentStatus</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>/Device/SubDevice[10]/Modules[6]</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>RunningStatus</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>BITFIELD</t>
+    <t>PRESENT_STATUS</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>E_DISABLED</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>E_ENABLED</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>E_NOT_PRESENT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>E_PRESENT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>E_INVALID</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>E_VALID</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>E_DISCONNECTED</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>E_AUTHENTICATING</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>E_AUTHENTICATION_FAILED</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>E_CONNECTED</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Present</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Not Present</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Disconnected</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Authenticating</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Authentication Failed</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Connected</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -616,151 +652,151 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>44</v>
-      </c>
       <c r="C2" s="3" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="E2" s="3">
         <v>1</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="E3" s="3">
         <v>1</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="E4" s="3">
         <v>1</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="E5" s="3">
         <v>1</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="E6" s="3">
         <v>1</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="E7" s="3">
         <v>1</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="E8" s="3">
         <v>1</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -786,7 +822,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="29.75" customWidth="1"/>
@@ -811,7 +847,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>17</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -819,10 +855,10 @@
         <v>0</v>
       </c>
       <c r="C3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D3" t="s">
         <v>16</v>
-      </c>
-      <c r="D3" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -830,42 +866,42 @@
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="D4" t="s">
-        <v>20</v>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>18</v>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6" t="s">
+        <v>44</v>
+      </c>
+      <c r="D6" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="D7" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B8">
-        <v>1</v>
-      </c>
-      <c r="C8" t="s">
-        <v>22</v>
-      </c>
-      <c r="D8" t="s">
-        <v>24</v>
+        <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
@@ -873,7 +909,10 @@
         <v>0</v>
       </c>
       <c r="C10" t="s">
-        <v>26</v>
+        <v>46</v>
+      </c>
+      <c r="D10" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
@@ -881,23 +920,59 @@
         <v>1</v>
       </c>
       <c r="C11" t="s">
-        <v>27</v>
+        <v>47</v>
+      </c>
+      <c r="D11" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B12">
-        <v>2</v>
-      </c>
-      <c r="C12" t="s">
-        <v>28</v>
+      <c r="A12" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B13">
+        <v>0</v>
+      </c>
+      <c r="C13" t="s">
+        <v>48</v>
+      </c>
+      <c r="D13" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>49</v>
+      </c>
+      <c r="D14" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B15">
+        <v>2</v>
+      </c>
+      <c r="C15" t="s">
+        <v>50</v>
+      </c>
+      <c r="D15" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B16">
         <v>3</v>
       </c>
-      <c r="C13" t="s">
-        <v>29</v>
+      <c r="C16" t="s">
+        <v>51</v>
+      </c>
+      <c r="D16" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>